<commit_message>
Siste oppdatering før jeg leverer prosjektet.
</commit_message>
<xml_diff>
--- a/Vedlegg 2 - Timeliste/Timeliste.xlsx
+++ b/Vedlegg 2 - Timeliste/Timeliste.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitLab\tisip_sisteaar\Avsluttende prosjekt\Rapport\Timeliste\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitLab\tisip_sisteaar\Avsluttende prosjekt\Rapport\Sikker kommunikasjon og sertifikathåndtering i byggautomasjon med Tailscale og OPC UA\Vedlegg 2 - Timeliste\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72F1C914-6C09-4A8E-A525-165C064684F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C45A2969-5630-4438-96EE-7E2833F8F0BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21090" yWindow="3375" windowWidth="28800" windowHeight="15555" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16260" yWindow="2145" windowWidth="21600" windowHeight="11505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="20">
   <si>
     <t>Dato</t>
   </si>
@@ -90,6 +90,9 @@
   </si>
   <si>
     <t>Skrive på rapporten, jobbe med referanser</t>
+  </si>
+  <si>
+    <t>Gjjøre ferdig rapport, levere den inn</t>
   </si>
 </sst>
 </file>
@@ -310,18 +313,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -329,34 +323,39 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -674,16 +673,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="2"/>
+      <c r="C1" s="22"/>
     </row>
     <row r="3" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="3"/>
+      <c r="C3" s="21"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -695,628 +694,628 @@
       <c r="C5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="15">
+      <c r="A6" s="11">
         <v>9</v>
       </c>
-      <c r="B6" s="21">
+      <c r="B6" s="17">
         <v>45712</v>
       </c>
-      <c r="C6" s="8">
-        <v>7.5</v>
-      </c>
-      <c r="D6" s="9" t="s">
+      <c r="C6" s="5">
+        <v>7.5</v>
+      </c>
+      <c r="D6" s="6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="16"/>
-      <c r="B7" s="22">
+      <c r="A7" s="12"/>
+      <c r="B7" s="18">
         <v>45713</v>
       </c>
-      <c r="C7" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D7" s="12" t="s">
+      <c r="C7">
+        <v>7.5</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="16"/>
-      <c r="B8" s="22">
+      <c r="A8" s="12"/>
+      <c r="B8" s="18">
         <v>45714</v>
       </c>
-      <c r="C8" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D8" s="12" t="s">
+      <c r="C8">
+        <v>7.5</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="16"/>
-      <c r="B9" s="22">
+      <c r="A9" s="12"/>
+      <c r="B9" s="18">
         <v>45715</v>
       </c>
-      <c r="C9" s="11">
+      <c r="C9">
         <v>4</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="8" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="17"/>
-      <c r="B10" s="23">
+      <c r="A10" s="13"/>
+      <c r="B10" s="19">
         <v>45716</v>
       </c>
-      <c r="C10" s="24">
+      <c r="C10" s="20">
         <v>3</v>
       </c>
-      <c r="D10" s="14" t="s">
+      <c r="D10" s="10" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="18">
+      <c r="A11" s="14">
         <v>10</v>
       </c>
-      <c r="B11" s="21">
+      <c r="B11" s="17">
         <v>45719</v>
       </c>
-      <c r="C11" s="8">
-        <v>7.5</v>
-      </c>
-      <c r="D11" s="9" t="s">
+      <c r="C11" s="5">
+        <v>7.5</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="19"/>
-      <c r="B12" s="22">
+      <c r="A12" s="15"/>
+      <c r="B12" s="18">
         <v>45720</v>
       </c>
-      <c r="C12" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D12" s="12" t="s">
+      <c r="C12">
+        <v>7.5</v>
+      </c>
+      <c r="D12" s="8" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="19"/>
-      <c r="B13" s="22">
+      <c r="A13" s="15"/>
+      <c r="B13" s="18">
         <v>45721</v>
       </c>
-      <c r="C13" s="11">
+      <c r="C13">
         <v>3</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="8" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="19"/>
-      <c r="B14" s="22">
+      <c r="A14" s="15"/>
+      <c r="B14" s="18">
         <v>45722</v>
       </c>
-      <c r="C14" s="11">
+      <c r="C14">
         <v>10</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="D14" s="8" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="20"/>
-      <c r="B15" s="23">
-        <v>45723</v>
-      </c>
-      <c r="C15" s="13">
-        <v>7.5</v>
-      </c>
-      <c r="D15" s="14" t="s">
+      <c r="A15" s="16"/>
+      <c r="B15" s="19">
+        <v>45724</v>
+      </c>
+      <c r="C15" s="9">
+        <v>7.5</v>
+      </c>
+      <c r="D15" s="10" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="18">
+      <c r="A16" s="14">
         <v>11</v>
       </c>
-      <c r="B16" s="21">
+      <c r="B16" s="17">
         <v>45726</v>
       </c>
-      <c r="C16" s="8">
-        <v>7.5</v>
-      </c>
-      <c r="D16" s="9" t="s">
+      <c r="C16" s="5">
+        <v>7.5</v>
+      </c>
+      <c r="D16" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="19"/>
-      <c r="B17" s="22">
+      <c r="A17" s="15"/>
+      <c r="B17" s="18">
         <v>45727</v>
       </c>
-      <c r="C17" s="11">
+      <c r="C17">
         <v>5</v>
       </c>
-      <c r="D17" s="12" t="s">
+      <c r="D17" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="19"/>
-      <c r="B18" s="22">
+      <c r="A18" s="15"/>
+      <c r="B18" s="18">
         <v>45728</v>
       </c>
-      <c r="C18" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D18" s="12" t="s">
+      <c r="C18">
+        <v>7.5</v>
+      </c>
+      <c r="D18" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="19"/>
-      <c r="B19" s="22">
+      <c r="A19" s="15"/>
+      <c r="B19" s="18">
         <v>45729</v>
       </c>
-      <c r="C19" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D19" s="12" t="s">
+      <c r="C19">
+        <v>7.5</v>
+      </c>
+      <c r="D19" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="20"/>
-      <c r="B20" s="23">
+      <c r="A20" s="16"/>
+      <c r="B20" s="19">
         <v>45730</v>
       </c>
-      <c r="C20" s="13">
-        <v>7.5</v>
-      </c>
-      <c r="D20" s="14" t="s">
+      <c r="C20" s="9">
+        <v>7.5</v>
+      </c>
+      <c r="D20" s="10" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="18">
+      <c r="A21" s="14">
         <v>12</v>
       </c>
-      <c r="B21" s="21">
+      <c r="B21" s="17">
         <v>45733</v>
       </c>
-      <c r="C21" s="8">
-        <v>7.5</v>
-      </c>
-      <c r="D21" s="9" t="s">
+      <c r="C21" s="5">
+        <v>7.5</v>
+      </c>
+      <c r="D21" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="19"/>
-      <c r="B22" s="22">
+      <c r="A22" s="15"/>
+      <c r="B22" s="18">
         <v>45734</v>
       </c>
-      <c r="C22" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D22" s="12" t="s">
+      <c r="C22">
+        <v>7.5</v>
+      </c>
+      <c r="D22" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="19"/>
-      <c r="B23" s="22">
+      <c r="A23" s="15"/>
+      <c r="B23" s="18">
         <v>45735</v>
       </c>
-      <c r="C23" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D23" s="12" t="s">
+      <c r="C23">
+        <v>7.5</v>
+      </c>
+      <c r="D23" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="19"/>
-      <c r="B24" s="22">
+      <c r="A24" s="15"/>
+      <c r="B24" s="18">
         <v>45736</v>
       </c>
-      <c r="C24" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D24" s="12" t="s">
+      <c r="C24">
+        <v>7.5</v>
+      </c>
+      <c r="D24" s="8" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="20"/>
-      <c r="B25" s="23">
+      <c r="A25" s="16"/>
+      <c r="B25" s="19">
         <v>45737</v>
       </c>
-      <c r="C25" s="13">
-        <v>7.5</v>
-      </c>
-      <c r="D25" s="14" t="s">
+      <c r="C25" s="9">
+        <v>7.5</v>
+      </c>
+      <c r="D25" s="10" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="18">
+      <c r="A26" s="14">
         <v>13</v>
       </c>
-      <c r="B26" s="21">
+      <c r="B26" s="17">
         <v>45740</v>
       </c>
-      <c r="C26" s="8">
-        <v>7.5</v>
-      </c>
-      <c r="D26" s="9" t="s">
+      <c r="C26" s="5">
+        <v>7.5</v>
+      </c>
+      <c r="D26" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="19"/>
-      <c r="B27" s="22">
+      <c r="A27" s="15"/>
+      <c r="B27" s="18">
         <v>45741</v>
       </c>
-      <c r="C27" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D27" s="12" t="s">
+      <c r="C27">
+        <v>7.5</v>
+      </c>
+      <c r="D27" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="19"/>
-      <c r="B28" s="22">
+      <c r="A28" s="15"/>
+      <c r="B28" s="18">
         <v>45742</v>
       </c>
-      <c r="C28" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D28" s="12" t="s">
+      <c r="C28">
+        <v>7.5</v>
+      </c>
+      <c r="D28" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="19"/>
-      <c r="B29" s="22">
+      <c r="A29" s="15"/>
+      <c r="B29" s="18">
         <v>45743</v>
       </c>
-      <c r="C29" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D29" s="12" t="s">
+      <c r="C29">
+        <v>7.5</v>
+      </c>
+      <c r="D29" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="20"/>
-      <c r="B30" s="23">
+      <c r="A30" s="16"/>
+      <c r="B30" s="19">
         <v>45744</v>
       </c>
-      <c r="C30" s="13">
+      <c r="C30" s="9">
         <v>6</v>
       </c>
-      <c r="D30" s="14" t="s">
+      <c r="D30" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="18">
+      <c r="A31" s="14">
         <v>14</v>
       </c>
-      <c r="B31" s="21">
+      <c r="B31" s="17">
         <v>45747</v>
       </c>
-      <c r="C31" s="8">
-        <v>7.5</v>
-      </c>
-      <c r="D31" s="9" t="s">
+      <c r="C31" s="5">
+        <v>7.5</v>
+      </c>
+      <c r="D31" s="6" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="19"/>
-      <c r="B32" s="22">
+      <c r="A32" s="15"/>
+      <c r="B32" s="18">
         <v>45748</v>
       </c>
-      <c r="C32" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D32" s="12" t="s">
+      <c r="C32">
+        <v>7.5</v>
+      </c>
+      <c r="D32" s="8" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="19"/>
-      <c r="B33" s="22">
+      <c r="A33" s="15"/>
+      <c r="B33" s="18">
         <v>45749</v>
       </c>
-      <c r="C33" s="11">
+      <c r="C33">
         <v>5</v>
       </c>
-      <c r="D33" s="12" t="s">
+      <c r="D33" s="8" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="19"/>
-      <c r="B34" s="22">
+      <c r="A34" s="15"/>
+      <c r="B34" s="18">
         <v>45750</v>
       </c>
-      <c r="C34" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D34" s="12" t="s">
+      <c r="C34">
+        <v>7.5</v>
+      </c>
+      <c r="D34" s="8" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="20"/>
-      <c r="B35" s="23">
+      <c r="A35" s="16"/>
+      <c r="B35" s="19">
         <v>45751</v>
       </c>
-      <c r="C35" s="13">
-        <v>7.5</v>
-      </c>
-      <c r="D35" s="14" t="s">
+      <c r="C35" s="9">
+        <v>7.5</v>
+      </c>
+      <c r="D35" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="18">
-        <v>15</v>
-      </c>
-      <c r="B36" s="21">
+      <c r="A36" s="14">
+        <v>15</v>
+      </c>
+      <c r="B36" s="17">
         <v>45754</v>
       </c>
-      <c r="C36" s="8">
-        <v>7.5</v>
-      </c>
-      <c r="D36" s="9" t="s">
+      <c r="C36" s="5">
+        <v>7.5</v>
+      </c>
+      <c r="D36" s="6" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="19"/>
-      <c r="B37" s="22">
+      <c r="A37" s="15"/>
+      <c r="B37" s="18">
         <v>45755</v>
       </c>
-      <c r="C37" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D37" s="12" t="s">
+      <c r="C37">
+        <v>7.5</v>
+      </c>
+      <c r="D37" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="19"/>
-      <c r="B38" s="22">
+      <c r="A38" s="15"/>
+      <c r="B38" s="18">
         <v>45756</v>
       </c>
-      <c r="C38" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D38" s="12" t="s">
+      <c r="C38">
+        <v>7.5</v>
+      </c>
+      <c r="D38" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="19"/>
-      <c r="B39" s="22">
+      <c r="A39" s="15"/>
+      <c r="B39" s="18">
         <v>45757</v>
       </c>
-      <c r="C39" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D39" s="12" t="s">
+      <c r="C39">
+        <v>7.5</v>
+      </c>
+      <c r="D39" s="8" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="20"/>
-      <c r="B40" s="23">
+      <c r="A40" s="16"/>
+      <c r="B40" s="19">
         <v>45758</v>
       </c>
-      <c r="C40" s="13">
-        <v>7.5</v>
-      </c>
-      <c r="D40" s="14" t="s">
+      <c r="C40" s="9">
+        <v>7.5</v>
+      </c>
+      <c r="D40" s="10" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="18">
+      <c r="A41" s="14">
         <v>16</v>
       </c>
-      <c r="B41" s="21">
+      <c r="B41" s="17">
         <v>45761</v>
       </c>
-      <c r="C41" s="8">
-        <v>7.5</v>
-      </c>
-      <c r="D41" s="9" t="s">
+      <c r="C41" s="5">
+        <v>7.5</v>
+      </c>
+      <c r="D41" s="6" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="19"/>
-      <c r="B42" s="22">
+      <c r="A42" s="15"/>
+      <c r="B42" s="18">
         <v>45762</v>
       </c>
-      <c r="C42" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D42" s="12" t="s">
+      <c r="C42">
+        <v>7.5</v>
+      </c>
+      <c r="D42" s="8" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="19"/>
-      <c r="B43" s="22">
+      <c r="A43" s="15"/>
+      <c r="B43" s="18">
         <v>45763</v>
       </c>
-      <c r="C43" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D43" s="12" t="s">
+      <c r="C43">
+        <v>7.5</v>
+      </c>
+      <c r="D43" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="19"/>
-      <c r="B44" s="22">
+      <c r="A44" s="15"/>
+      <c r="B44" s="18">
         <v>45764</v>
       </c>
-      <c r="C44" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D44" s="12" t="s">
+      <c r="C44">
+        <v>7.5</v>
+      </c>
+      <c r="D44" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="20"/>
-      <c r="B45" s="23">
+      <c r="A45" s="16"/>
+      <c r="B45" s="19">
         <v>45765</v>
       </c>
-      <c r="C45" s="13">
-        <v>7.5</v>
-      </c>
-      <c r="D45" s="14" t="s">
+      <c r="C45" s="9">
+        <v>7.5</v>
+      </c>
+      <c r="D45" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="18">
+      <c r="A46" s="14">
         <v>17</v>
       </c>
-      <c r="B46" s="21">
-        <v>45768</v>
-      </c>
-      <c r="C46" s="8">
+      <c r="B46" s="17">
+        <v>45766</v>
+      </c>
+      <c r="C46" s="5">
         <v>5</v>
       </c>
-      <c r="D46" s="9" t="s">
+      <c r="D46" s="6" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="19"/>
-      <c r="B47" s="22">
+      <c r="A47" s="15"/>
+      <c r="B47" s="18">
         <v>45769</v>
       </c>
-      <c r="C47" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D47" s="12" t="s">
+      <c r="C47">
+        <v>7.5</v>
+      </c>
+      <c r="D47" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="19"/>
-      <c r="B48" s="22">
+      <c r="A48" s="15"/>
+      <c r="B48" s="18">
         <v>45770</v>
       </c>
-      <c r="C48" s="11">
+      <c r="C48">
         <v>4</v>
       </c>
-      <c r="D48" s="12" t="s">
+      <c r="D48" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="19"/>
-      <c r="B49" s="22">
+      <c r="A49" s="15"/>
+      <c r="B49" s="18">
         <v>45771</v>
       </c>
-      <c r="C49" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D49" s="12" t="s">
+      <c r="C49">
+        <v>7.5</v>
+      </c>
+      <c r="D49" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="20"/>
-      <c r="B50" s="23">
+      <c r="A50" s="16"/>
+      <c r="B50" s="19">
         <v>45772</v>
       </c>
-      <c r="C50" s="13">
-        <v>7.5</v>
-      </c>
-      <c r="D50" s="14" t="s">
+      <c r="C50" s="9">
+        <v>7.5</v>
+      </c>
+      <c r="D50" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="18">
+      <c r="A51" s="14">
         <v>18</v>
       </c>
-      <c r="B51" s="10">
-        <v>45775</v>
-      </c>
-      <c r="C51" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D51" s="12" t="s">
+      <c r="B51" s="7">
+        <v>45774</v>
+      </c>
+      <c r="C51">
+        <v>7.5</v>
+      </c>
+      <c r="D51" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="19"/>
-      <c r="B52" s="10">
+      <c r="A52" s="15"/>
+      <c r="B52" s="7">
         <v>45776</v>
       </c>
-      <c r="C52" s="11">
-        <v>7.5</v>
-      </c>
-      <c r="D52" s="12" t="s">
+      <c r="C52">
+        <v>7.5</v>
+      </c>
+      <c r="D52" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="19"/>
-      <c r="B53" s="10">
-        <v>45777</v>
-      </c>
-      <c r="C53" s="11">
+      <c r="A53" s="15"/>
+      <c r="B53" s="7">
+        <v>45778</v>
+      </c>
+      <c r="C53">
         <v>3</v>
       </c>
-      <c r="D53" s="12" t="s">
+      <c r="D53" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="20"/>
-      <c r="B54" s="10">
-        <v>45778</v>
-      </c>
-      <c r="C54" s="11">
-        <v>3</v>
-      </c>
-      <c r="D54" s="12" t="s">
-        <v>15</v>
+      <c r="A54" s="16"/>
+      <c r="B54" s="7">
+        <v>45795</v>
+      </c>
+      <c r="C54">
+        <v>7.5</v>
+      </c>
+      <c r="D54" s="8" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="5"/>
-      <c r="B55" s="6" t="s">
+      <c r="A55" s="2"/>
+      <c r="B55" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C55" s="6">
+      <c r="C55" s="3">
         <f>SUM(C11:C54)</f>
-        <v>306.5</v>
-      </c>
-      <c r="D55" s="7"/>
+        <v>311</v>
+      </c>
+      <c r="D55" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>